<commit_message>
feat(v1.1.0): interfaz web interactiva, memoria multi-colegio, gestor dinamico de nominas Excel, OAuth 2.0 y scripts de instalacion 1-clic
</commit_message>
<xml_diff>
--- a/output/Cronograma_Entrevistas_Apoderados_2026.xlsx
+++ b/output/Cronograma_Entrevistas_Apoderados_2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entrevistas Apoderados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma Entrevistas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,18 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7E34"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -63,14 +75,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6FAFE"/>
-        <bgColor rgb="00F6FAFE"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00EAF3FB"/>
+        <bgColor rgb="00EAF3FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -100,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -117,11 +129,23 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,33 +512,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COLEGIO LUIS PASTEUR ANEXO - CRONOGRAMA DE ENTREVISTAS DE APODERADOS 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>COLEGIO LUIS PASTEUR ANEXO — CRONOGRAMA DE ENTREVISTAS DE APODERADOS 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Profesora Margarita Miranda B. | Jefatura 5° Básico A y Asignaturas</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="25" customHeight="1">
+          <t>Gestión de Asignatura y Jefatura de Curso | Profesora Margarita Miranda B. | Sistema EduDocente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>N°</t>
@@ -542,16 +569,26 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Fecha entrevista</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Hora de entrevista</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="21" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -577,57 +614,77 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 07 de octubre</t>
+          <t>Miércoles</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="n">
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>María Reyes</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>mariareyessanti.14@gmail.com</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Reyes Cabrera, Catalina Amanda</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 07 de octubre</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="21" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Aurora Celin / Familia Celin Mosquera</t>
+          <t>Aurora Celin / Familia Celin</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -647,51 +704,71 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 07 de octubre</t>
+          <t>Miércoles</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="4" t="n">
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="21" customHeight="1">
+      <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Cecilia Riquelme Cartagena</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>ceci.riquelme.cartagena@gmail.com</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Segovia Riquelme, Marcelo Leonardo</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 07 de octubre</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="21" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -717,51 +794,71 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 07 de octubre</t>
+          <t>Miércoles</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="n">
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="21" customHeight="1">
+      <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Luz Elena Guerrero</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>luzeg782511@gmail.com</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Restrepo Guerrero, Luis David</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 07 de octubre</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="21" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -787,335 +884,440 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 07 de octubre</t>
+          <t>Miércoles</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="n">
+          <t>07 de octubre</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Mella Navarrete (Sra. Mella)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>mella.navarrete.m@gmail.com</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Aravena Mella, Martín Andree</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Marcia Elizabeth Pacheco Pacheco</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Marcia Elizabeth Pacheco</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>marciaelizabethpachecopacheco@gmail.com</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Flores Pacheco, Hamandha Sophia</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="n">
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Osvaldo González Correa</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>osvaldo.gonzalez.correa@gmail.com</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>González Ibáñez, Amanda Trinidad</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="n">
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>David Ignacio Herrera Rojas</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>davidignacioherrerarojas@gmail.com</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Herrera Díaz, Paz Anaís</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="n">
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Valentina Constanza Aguayo Trejo</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Valentina Constanza Aguayo</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>valentinacaguayo7@gmail.com</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Leyton Aguayo, Gabriel Andrés</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="6" t="n">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Familia Morales Silva (Claro de Luna)</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Familia Morales Silva</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>clarodeluna_1980@htmail.com</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Morales Silva, Danilo Cristián</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>5° Básico A</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="6" t="n">
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Fabiola Mora C.</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>fabiola.mora.c@gmail.com</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Ibarra Oyarzún, Benjamín Ricardo</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>8° Básico A</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="6" t="n">
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Verónica Urrutia (Verito Eleniz)</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Verónica Urrutia</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>veritoeleniz2013@gmail.com</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Lobos Urrutia, Eleniz Javiera Lía</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>8° Básico A</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="A20" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Carana M. / Familia Arana</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>caranamza@gmail.com</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Oliva Arana, Thiago Yared</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>8° Básico A</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Miércoles 14 de octubre</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>13:55 a 14:40 hrs</t>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>14 de octubre</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>13:55 a 14:40 hrs</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="I5:I71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Confirmado,Pendiente,Reprogramado,Inasistencia"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>